<commit_message>
add 1k5 and 1nF
</commit_message>
<xml_diff>
--- a/Librairies/TEP-AltiumLib-Passives-RLC.xlsx
+++ b/Librairies/TEP-AltiumLib-Passives-RLC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lecegeplimoilou-my.sharepoint.com/personal/kevin_cotton_cegeplimoilou_ca/Documents/_Cours-TGE/Altium/243-TEP_Altium-Lib/Librairies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1419" documentId="13_ncr:1_{550D3E46-E4B6-4165-A45B-7D583CCE157E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B78C59A-30BB-44EE-8878-108D214892C5}"/>
+  <xr:revisionPtr revIDLastSave="1440" documentId="13_ncr:1_{550D3E46-E4B6-4165-A45B-7D583CCE157E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11D1E836-EED1-4A21-BDD9-16E427D43CEB}"/>
   <bookViews>
-    <workbookView xWindow="3108" yWindow="588" windowWidth="18636" windowHeight="11616" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="636" windowWidth="19380" windowHeight="9516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cap" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1225" uniqueCount="470">
   <si>
     <t>Comment</t>
   </si>
@@ -291,9 +291,6 @@
     <t>Digikey</t>
   </si>
   <si>
-    <t>Digi-Key</t>
-  </si>
-  <si>
     <t>Res 2k2 1% 0402</t>
   </si>
   <si>
@@ -1420,6 +1417,42 @@
   </si>
   <si>
     <t>TEP-AltiumLib-Passives.PcbLib</t>
+  </si>
+  <si>
+    <t>RES047</t>
+  </si>
+  <si>
+    <t>Res 1k5 1% 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-071k5L</t>
+  </si>
+  <si>
+    <t>1k5</t>
+  </si>
+  <si>
+    <t>C114759</t>
+  </si>
+  <si>
+    <t>311-1.50KLRCT-ND</t>
+  </si>
+  <si>
+    <t>CAP027</t>
+  </si>
+  <si>
+    <t>CAP CER 1nF 50V X7R 0402</t>
+  </si>
+  <si>
+    <t>CC0402KRX7R9BB102</t>
+  </si>
+  <si>
+    <t>1nF</t>
+  </si>
+  <si>
+    <t>C106205</t>
+  </si>
+  <si>
+    <t>311-1036-1-ND</t>
   </si>
 </sst>
 </file>
@@ -1488,7 +1521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1513,6 +1546,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1795,7 +1829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -1819,10 +1853,10 @@
         <v>5</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>313</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>314</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>0</v>
@@ -1846,7 +1880,7 @@
         <v>4</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>15</v>
@@ -1867,10 +1901,10 @@
         <v>42</v>
       </c>
       <c r="R1" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="S1" s="13" t="s">
         <v>93</v>
-      </c>
-      <c r="S1" s="13" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
@@ -1878,22 +1912,22 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E2" t="s">
         <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I2" t="s">
         <v>11</v>
@@ -1908,19 +1942,19 @@
         <v>21</v>
       </c>
       <c r="M2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N2" t="s">
         <v>29</v>
       </c>
       <c r="O2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P2" t="s">
         <v>44</v>
       </c>
       <c r="Q2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
@@ -1928,22 +1962,22 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E3" t="s">
         <v>67</v>
       </c>
       <c r="F3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I3" t="s">
         <v>11</v>
@@ -1958,19 +1992,19 @@
         <v>21</v>
       </c>
       <c r="M3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N3" t="s">
         <v>30</v>
       </c>
       <c r="O3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P3" t="s">
         <v>44</v>
       </c>
       <c r="Q3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
@@ -1978,22 +2012,22 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E4" t="s">
         <v>73</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G4" t="s">
         <v>74</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I4" t="s">
         <v>69</v>
@@ -2008,19 +2042,19 @@
         <v>21</v>
       </c>
       <c r="M4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N4" t="s">
         <v>79</v>
       </c>
       <c r="O4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P4" t="s">
         <v>44</v>
       </c>
       <c r="Q4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.3">
@@ -2028,23 +2062,23 @@
         <v>24</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E5" t="s">
+        <v>352</v>
+      </c>
+      <c r="F5" t="s">
         <v>353</v>
-      </c>
-      <c r="F5" t="s">
-        <v>354</v>
       </c>
       <c r="G5" t="s">
         <v>75</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I5" t="s">
         <v>70</v>
@@ -2059,19 +2093,19 @@
         <v>21</v>
       </c>
       <c r="M5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N5" t="s">
         <v>79</v>
       </c>
       <c r="O5" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P5" t="s">
         <v>44</v>
       </c>
       <c r="Q5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.3">
@@ -2079,23 +2113,23 @@
         <v>71</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G6" t="s">
         <v>76</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I6" t="s">
         <v>70</v>
@@ -2110,19 +2144,19 @@
         <v>21</v>
       </c>
       <c r="M6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N6" s="8" t="s">
         <v>80</v>
       </c>
       <c r="O6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P6" t="s">
         <v>44</v>
       </c>
       <c r="Q6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.3">
@@ -2130,25 +2164,25 @@
         <v>72</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G7" t="s">
         <v>77</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I7" t="s">
         <v>11</v>
       </c>
       <c r="J7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K7" t="s">
         <v>13</v>
@@ -2157,39 +2191,39 @@
         <v>21</v>
       </c>
       <c r="M7" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N7" t="s">
         <v>29</v>
       </c>
       <c r="O7" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P7" t="s">
         <v>44</v>
       </c>
       <c r="Q7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E8" t="s">
         <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I8" t="s">
         <v>11</v>
@@ -2204,42 +2238,42 @@
         <v>21</v>
       </c>
       <c r="M8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N8" t="s">
         <v>30</v>
       </c>
       <c r="O8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P8" t="s">
         <v>44</v>
       </c>
       <c r="Q8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E9" t="s">
         <v>67</v>
       </c>
       <c r="F9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I9" t="s">
         <v>11</v>
@@ -2254,42 +2288,42 @@
         <v>21</v>
       </c>
       <c r="M9" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N9" t="s">
         <v>79</v>
       </c>
       <c r="O9" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P9" t="s">
         <v>44</v>
       </c>
       <c r="Q9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" t="s">
+        <v>249</v>
+      </c>
+      <c r="E10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F10" t="s">
+        <v>112</v>
+      </c>
+      <c r="G10" t="s">
+        <v>115</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I10" t="s">
         <v>114</v>
-      </c>
-      <c r="D10" t="s">
-        <v>250</v>
-      </c>
-      <c r="E10" t="s">
-        <v>112</v>
-      </c>
-      <c r="F10" t="s">
-        <v>113</v>
-      </c>
-      <c r="G10" t="s">
-        <v>116</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="I10" t="s">
-        <v>115</v>
       </c>
       <c r="J10" t="s">
         <v>12</v>
@@ -2301,45 +2335,45 @@
         <v>21</v>
       </c>
       <c r="M10" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N10" t="s">
         <v>30</v>
       </c>
       <c r="O10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P10" t="s">
         <v>44</v>
       </c>
       <c r="Q10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E11" t="s">
         <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I11" t="s">
         <v>11</v>
       </c>
       <c r="J11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K11" t="s">
         <v>13</v>
@@ -2348,42 +2382,42 @@
         <v>21</v>
       </c>
       <c r="M11" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N11" t="s">
         <v>29</v>
       </c>
       <c r="O11" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P11" t="s">
         <v>44</v>
       </c>
       <c r="Q11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="E12" t="s">
+        <v>111</v>
+      </c>
+      <c r="F12" t="s">
+        <v>356</v>
+      </c>
+      <c r="G12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>356</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="E12" t="s">
-        <v>112</v>
-      </c>
-      <c r="F12" t="s">
-        <v>357</v>
-      </c>
-      <c r="G12" t="s">
-        <v>163</v>
-      </c>
       <c r="H12" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I12" t="s">
         <v>11</v>
@@ -2398,49 +2432,49 @@
         <v>21</v>
       </c>
       <c r="M12" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N12" t="s">
         <v>79</v>
       </c>
       <c r="O12" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P12" t="s">
         <v>44</v>
       </c>
       <c r="Q12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>164</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>165</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I13" t="s">
         <v>11</v>
       </c>
       <c r="J13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K13" t="s">
         <v>13</v>
@@ -2449,43 +2483,43 @@
         <v>21</v>
       </c>
       <c r="M13" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N13" s="6" t="s">
         <v>30</v>
       </c>
       <c r="O13" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I14" t="s">
         <v>11</v>
       </c>
       <c r="J14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K14" t="s">
         <v>13</v>
@@ -2494,39 +2528,39 @@
         <v>21</v>
       </c>
       <c r="M14" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N14" t="s">
         <v>80</v>
       </c>
       <c r="O14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E15" t="s">
         <v>67</v>
       </c>
       <c r="F15" t="s">
+        <v>189</v>
+      </c>
+      <c r="G15" t="s">
         <v>190</v>
       </c>
-      <c r="G15" t="s">
-        <v>191</v>
-      </c>
       <c r="H15" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I15" t="s">
         <v>11</v>
       </c>
       <c r="J15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K15" t="s">
         <v>13</v>
@@ -2535,45 +2569,45 @@
         <v>21</v>
       </c>
       <c r="M15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N15" t="s">
         <v>29</v>
       </c>
       <c r="O15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P15" t="s">
         <v>44</v>
       </c>
       <c r="Q15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E16" t="s">
         <v>67</v>
       </c>
       <c r="F16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I16" t="s">
         <v>11</v>
       </c>
       <c r="J16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K16" t="s">
         <v>13</v>
@@ -2582,42 +2616,42 @@
         <v>21</v>
       </c>
       <c r="M16" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N16" t="s">
         <v>29</v>
       </c>
       <c r="O16" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P16" t="s">
         <v>44</v>
       </c>
       <c r="Q16" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>195</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E17" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" t="s">
         <v>194</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>196</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="E17" t="s">
-        <v>112</v>
-      </c>
-      <c r="F17" t="s">
-        <v>195</v>
       </c>
       <c r="G17" t="s">
         <v>74</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J17" t="s">
         <v>78</v>
@@ -2629,39 +2663,39 @@
         <v>21</v>
       </c>
       <c r="M17" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N17" t="s">
         <v>29</v>
       </c>
       <c r="O17" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P17" t="s">
         <v>44</v>
       </c>
       <c r="Q17" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>199</v>
-      </c>
       <c r="D18" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E18" t="s">
         <v>67</v>
       </c>
       <c r="F18" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I18" t="s">
         <v>11</v>
@@ -2676,45 +2710,45 @@
         <v>21</v>
       </c>
       <c r="M18" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N18" t="s">
         <v>29</v>
       </c>
       <c r="O18" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P18" t="s">
         <v>44</v>
       </c>
       <c r="Q18" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D19" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E19" t="s">
         <v>67</v>
       </c>
       <c r="F19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G19" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I19" t="s">
         <v>11</v>
       </c>
       <c r="J19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K19" t="s">
         <v>13</v>
@@ -2723,45 +2757,45 @@
         <v>21</v>
       </c>
       <c r="M19" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N19" t="s">
         <v>29</v>
       </c>
       <c r="O19" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P19" t="s">
         <v>44</v>
       </c>
       <c r="Q19" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D20" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E20" t="s">
         <v>67</v>
       </c>
       <c r="F20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I20" t="s">
         <v>11</v>
       </c>
       <c r="J20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K20" t="s">
         <v>13</v>
@@ -2770,39 +2804,39 @@
         <v>21</v>
       </c>
       <c r="M20" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N20" t="s">
         <v>29</v>
       </c>
       <c r="O20" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P20" t="s">
         <v>44</v>
       </c>
       <c r="Q20" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G21" t="s">
         <v>75</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I21" t="s">
         <v>69</v>
@@ -2817,86 +2851,86 @@
         <v>21</v>
       </c>
       <c r="M21" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N21" t="s">
         <v>79</v>
       </c>
       <c r="O21" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P21" t="s">
         <v>44</v>
       </c>
       <c r="Q21" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>319</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>321</v>
-      </c>
       <c r="E22" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F22" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G22" t="s">
         <v>76</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I22" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="J22" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K22" t="s">
         <v>13</v>
       </c>
       <c r="L22" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="M22" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N22" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="O22" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P22" t="s">
         <v>44</v>
       </c>
       <c r="Q22" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>364</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>366</v>
-      </c>
       <c r="E23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F23" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G23" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I23" t="s">
         <v>70</v>
@@ -2911,39 +2945,39 @@
         <v>21</v>
       </c>
       <c r="M23" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N23" t="s">
         <v>30</v>
       </c>
       <c r="O23" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P23" t="s">
         <v>44</v>
       </c>
       <c r="Q23" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>421</v>
+      </c>
+      <c r="B24" t="s">
         <v>422</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>423</v>
       </c>
-      <c r="C24" t="s">
-        <v>424</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G24" t="s">
         <v>75</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I24" t="s">
         <v>11</v>
@@ -2958,30 +2992,30 @@
         <v>21</v>
       </c>
       <c r="M24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N24" s="8" t="s">
         <v>80</v>
       </c>
       <c r="O24" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B25" t="s">
+        <v>425</v>
+      </c>
+      <c r="C25" t="s">
         <v>426</v>
       </c>
-      <c r="C25" t="s">
-        <v>427</v>
-      </c>
       <c r="D25" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="G25" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I25" t="s">
         <v>11</v>
@@ -2993,30 +3027,30 @@
         <v>21</v>
       </c>
       <c r="M25" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N25" t="s">
         <v>30</v>
       </c>
       <c r="O25" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B26" t="s">
+        <v>427</v>
+      </c>
+      <c r="C26" t="s">
         <v>428</v>
       </c>
-      <c r="C26" t="s">
-        <v>429</v>
-      </c>
       <c r="D26" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G26" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="I26" t="s">
         <v>11</v>
@@ -3028,27 +3062,27 @@
         <v>21</v>
       </c>
       <c r="M26" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N26" t="s">
         <v>30</v>
       </c>
       <c r="O26" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B27" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C27" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D27" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="G27" t="s">
         <v>75</v>
@@ -3063,13 +3097,66 @@
         <v>21</v>
       </c>
       <c r="M27" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N27" t="s">
         <v>79</v>
       </c>
       <c r="O27" t="s">
-        <v>458</v>
+        <v>457</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>464</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>465</v>
+      </c>
+      <c r="E28" t="s">
+        <v>67</v>
+      </c>
+      <c r="F28" t="s">
+        <v>466</v>
+      </c>
+      <c r="G28" t="s">
+        <v>467</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I28" t="s">
+        <v>11</v>
+      </c>
+      <c r="J28" t="s">
+        <v>12</v>
+      </c>
+      <c r="K28" t="s">
+        <v>13</v>
+      </c>
+      <c r="L28" t="s">
+        <v>21</v>
+      </c>
+      <c r="M28" t="s">
+        <v>456</v>
+      </c>
+      <c r="N28" t="s">
+        <v>29</v>
+      </c>
+      <c r="O28" t="s">
+        <v>457</v>
+      </c>
+      <c r="P28" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>468</v>
+      </c>
+      <c r="R28" t="s">
+        <v>81</v>
+      </c>
+      <c r="S28" t="s">
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -3081,7 +3168,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0837104-CD0C-4055-94B3-0A98F94F86E8}">
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -3106,10 +3193,10 @@
         <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>313</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>314</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>0</v>
@@ -3133,7 +3220,7 @@
         <v>20</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>15</v>
@@ -3154,10 +3241,10 @@
         <v>42</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
@@ -3165,7 +3252,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>59</v>
@@ -3174,19 +3261,19 @@
         <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I2" t="s">
         <v>10</v>
       </c>
       <c r="J2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K2" t="s">
         <v>13</v>
@@ -3195,19 +3282,19 @@
         <v>25</v>
       </c>
       <c r="M2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P2" t="s">
         <v>44</v>
       </c>
       <c r="Q2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
@@ -3221,19 +3308,19 @@
         <v>67</v>
       </c>
       <c r="F3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G3" t="s">
         <v>35</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I3" t="s">
         <v>10</v>
       </c>
       <c r="J3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K3" t="s">
         <v>13</v>
@@ -3242,19 +3329,19 @@
         <v>25</v>
       </c>
       <c r="M3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P3" t="s">
         <v>44</v>
       </c>
       <c r="Q3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
@@ -3268,13 +3355,13 @@
         <v>67</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G4" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I4" t="s">
         <v>36</v>
@@ -3289,19 +3376,19 @@
         <v>25</v>
       </c>
       <c r="M4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P4" t="s">
         <v>44</v>
       </c>
       <c r="Q4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.3">
@@ -3315,13 +3402,13 @@
         <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G5" t="s">
         <v>35</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I5" t="s">
         <v>36</v>
@@ -3336,19 +3423,19 @@
         <v>25</v>
       </c>
       <c r="M5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O5" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P5" t="s">
         <v>44</v>
       </c>
       <c r="Q5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.3">
@@ -3356,7 +3443,7 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>56</v>
@@ -3380,19 +3467,19 @@
         <v>25</v>
       </c>
       <c r="M6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P6" t="s">
         <v>44</v>
       </c>
       <c r="Q6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.3">
@@ -3400,7 +3487,7 @@
         <v>49</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D7" t="s">
         <v>61</v>
@@ -3415,7 +3502,7 @@
         <v>64</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I7" t="s">
         <v>36</v>
@@ -3430,19 +3517,19 @@
         <v>25</v>
       </c>
       <c r="M7" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N7" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O7" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P7" t="s">
         <v>44</v>
       </c>
       <c r="Q7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.3">
@@ -3450,7 +3537,7 @@
         <v>50</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>62</v>
@@ -3459,13 +3546,13 @@
         <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G8" t="s">
         <v>65</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I8" t="s">
         <v>36</v>
@@ -3480,19 +3567,19 @@
         <v>25</v>
       </c>
       <c r="M8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>44</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.3">
@@ -3500,22 +3587,22 @@
         <v>51</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
         <v>67</v>
       </c>
       <c r="F9" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" t="s">
         <v>85</v>
       </c>
-      <c r="G9" t="s">
-        <v>86</v>
-      </c>
       <c r="H9" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I9" t="s">
         <v>36</v>
@@ -3530,25 +3617,25 @@
         <v>25</v>
       </c>
       <c r="M9" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N9" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O9" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>44</v>
       </c>
       <c r="Q9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.3">
@@ -3556,19 +3643,19 @@
         <v>52</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E10" t="s">
         <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I10" t="s">
         <v>36</v>
@@ -3583,25 +3670,25 @@
         <v>25</v>
       </c>
       <c r="M10" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N10" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>44</v>
       </c>
       <c r="Q10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="R10" t="s">
         <v>81</v>
       </c>
       <c r="S10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.3">
@@ -3609,19 +3696,19 @@
         <v>53</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E11" t="s">
         <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I11" t="s">
         <v>36</v>
@@ -3636,19 +3723,19 @@
         <v>25</v>
       </c>
       <c r="M11" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O11" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P11" t="s">
         <v>44</v>
       </c>
       <c r="Q11" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
@@ -3656,22 +3743,22 @@
         <v>54</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E12" t="s">
         <v>67</v>
       </c>
       <c r="F12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I12" t="s">
         <v>36</v>
@@ -3686,19 +3773,19 @@
         <v>25</v>
       </c>
       <c r="M12" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N12" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O12" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P12" t="s">
         <v>44</v>
       </c>
       <c r="Q12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.3">
@@ -3706,22 +3793,22 @@
         <v>55</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
         <v>67</v>
       </c>
       <c r="F13" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I13" t="s">
         <v>36</v>
@@ -3736,39 +3823,39 @@
         <v>25</v>
       </c>
       <c r="M13" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N13" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O13" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P13" t="s">
         <v>44</v>
       </c>
       <c r="Q13" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E14" t="s">
         <v>67</v>
       </c>
       <c r="F14" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I14" t="s">
         <v>36</v>
@@ -3783,48 +3870,48 @@
         <v>25</v>
       </c>
       <c r="M14" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O14" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P14" t="s">
         <v>44</v>
       </c>
       <c r="Q14" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B15" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E15" t="s">
         <v>67</v>
       </c>
       <c r="F15" t="s">
+        <v>295</v>
+      </c>
+      <c r="G15" t="s">
+        <v>172</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I15" t="s">
+        <v>173</v>
+      </c>
+      <c r="J15" t="s">
         <v>296</v>
-      </c>
-      <c r="G15" t="s">
-        <v>173</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="I15" t="s">
-        <v>174</v>
-      </c>
-      <c r="J15" t="s">
-        <v>297</v>
       </c>
       <c r="K15" t="s">
         <v>13</v>
@@ -3833,51 +3920,51 @@
         <v>25</v>
       </c>
       <c r="M15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P15" t="s">
         <v>44</v>
       </c>
       <c r="Q15" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="R15" t="s">
         <v>81</v>
       </c>
       <c r="S15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>176</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>178</v>
       </c>
       <c r="E16" t="s">
         <v>67</v>
       </c>
       <c r="F16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>64</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I16" t="s">
         <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K16" t="s">
         <v>13</v>
@@ -3886,48 +3973,48 @@
         <v>25</v>
       </c>
       <c r="M16" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O16" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P16" t="s">
         <v>44</v>
       </c>
       <c r="Q16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>181</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="D17" t="s">
         <v>182</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="D17" t="s">
-        <v>183</v>
       </c>
       <c r="E17" t="s">
         <v>67</v>
       </c>
       <c r="F17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I17" t="s">
         <v>10</v>
       </c>
       <c r="J17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K17" t="s">
         <v>13</v>
@@ -3936,39 +4023,39 @@
         <v>25</v>
       </c>
       <c r="M17" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N17" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O17" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P17" t="s">
         <v>44</v>
       </c>
       <c r="Q17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E18" t="s">
         <v>67</v>
       </c>
       <c r="F18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G18" t="s">
         <v>211</v>
       </c>
-      <c r="G18" t="s">
-        <v>212</v>
-      </c>
       <c r="H18" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I18" t="s">
         <v>36</v>
@@ -3983,45 +4070,45 @@
         <v>25</v>
       </c>
       <c r="M18" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N18" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O18" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P18" t="s">
         <v>44</v>
       </c>
       <c r="Q18" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>236</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="E19" t="s">
         <v>67</v>
       </c>
       <c r="F19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I19" t="s">
         <v>10</v>
       </c>
       <c r="J19" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K19" t="s">
         <v>13</v>
@@ -4030,54 +4117,54 @@
         <v>25</v>
       </c>
       <c r="M19" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N19" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O19" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P19" t="s">
         <v>44</v>
       </c>
       <c r="Q19" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="R19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="S19" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D20" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E20" t="s">
         <v>67</v>
       </c>
       <c r="F20" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J20" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K20" t="s">
         <v>13</v>
@@ -4086,48 +4173,48 @@
         <v>25</v>
       </c>
       <c r="M20" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O20" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P20" t="s">
         <v>44</v>
       </c>
       <c r="Q20" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D21" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="E21" t="s">
         <v>67</v>
       </c>
       <c r="F21" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K21" t="s">
         <v>13</v>
@@ -4136,48 +4223,48 @@
         <v>25</v>
       </c>
       <c r="M21" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O21" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P21" t="s">
         <v>44</v>
       </c>
       <c r="Q21" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D22" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E22" t="s">
         <v>67</v>
       </c>
       <c r="F22" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I22" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J22" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K22" t="s">
         <v>13</v>
@@ -4186,48 +4273,48 @@
         <v>25</v>
       </c>
       <c r="M22" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O22" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P22" t="s">
         <v>44</v>
       </c>
       <c r="Q22" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D23" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E23" t="s">
         <v>67</v>
       </c>
       <c r="F23" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J23" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K23" t="s">
         <v>13</v>
@@ -4236,48 +4323,48 @@
         <v>25</v>
       </c>
       <c r="M23" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O23" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P23" t="s">
         <v>44</v>
       </c>
       <c r="Q23" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D24" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E24" t="s">
         <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J24" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K24" t="s">
         <v>13</v>
@@ -4286,48 +4373,48 @@
         <v>25</v>
       </c>
       <c r="M24" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P24" t="s">
         <v>44</v>
       </c>
       <c r="Q24" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>285</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="B25" s="10" t="s">
-        <v>287</v>
-      </c>
       <c r="D25" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E25" t="s">
         <v>67</v>
       </c>
       <c r="F25" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>64</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J25" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K25" t="s">
         <v>13</v>
@@ -4336,48 +4423,48 @@
         <v>25</v>
       </c>
       <c r="M25" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O25" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P25" t="s">
         <v>44</v>
       </c>
       <c r="Q25" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D26" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E26" t="s">
         <v>67</v>
       </c>
       <c r="F26" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I26" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K26" t="s">
         <v>13</v>
@@ -4386,39 +4473,39 @@
         <v>25</v>
       </c>
       <c r="M26" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O26" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P26" t="s">
         <v>44</v>
       </c>
       <c r="Q26" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>290</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>292</v>
       </c>
       <c r="E27" t="s">
         <v>67</v>
       </c>
       <c r="F27" t="s">
+        <v>292</v>
+      </c>
+      <c r="G27" t="s">
         <v>293</v>
       </c>
-      <c r="G27" t="s">
-        <v>294</v>
-      </c>
       <c r="H27" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I27" t="s">
         <v>36</v>
@@ -4433,39 +4520,39 @@
         <v>25</v>
       </c>
       <c r="M27" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N27" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O27" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P27" t="s">
         <v>44</v>
       </c>
       <c r="Q27" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>314</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>315</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>316</v>
       </c>
       <c r="E28" t="s">
         <v>67</v>
       </c>
       <c r="F28" t="s">
+        <v>316</v>
+      </c>
+      <c r="G28" t="s">
         <v>317</v>
       </c>
-      <c r="G28" t="s">
-        <v>318</v>
-      </c>
       <c r="H28" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I28" t="s">
         <v>36</v>
@@ -4480,39 +4567,39 @@
         <v>25</v>
       </c>
       <c r="M28" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N28" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O28" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P28" t="s">
         <v>44</v>
       </c>
       <c r="Q28" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E29" t="s">
         <v>67</v>
       </c>
       <c r="F29" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I29" t="s">
         <v>36</v>
@@ -4527,45 +4614,45 @@
         <v>25</v>
       </c>
       <c r="M29" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N29" s="2" t="s">
         <v>37</v>
       </c>
       <c r="O29" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P29" t="s">
         <v>44</v>
       </c>
       <c r="Q29" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E30" t="s">
         <v>67</v>
       </c>
       <c r="F30" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I30" t="s">
         <v>10</v>
       </c>
       <c r="J30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K30" t="s">
         <v>13</v>
@@ -4574,45 +4661,45 @@
         <v>25</v>
       </c>
       <c r="M30" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N30" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O30" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P30" t="s">
         <v>44</v>
       </c>
       <c r="Q30" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D31" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E31" t="s">
         <v>67</v>
       </c>
       <c r="F31" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I31" t="s">
         <v>10</v>
       </c>
       <c r="J31" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K31" t="s">
         <v>13</v>
@@ -4621,45 +4708,45 @@
         <v>25</v>
       </c>
       <c r="M31" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N31" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O31" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P31" t="s">
         <v>44</v>
       </c>
       <c r="Q31" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D32" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E32" t="s">
         <v>67</v>
       </c>
       <c r="F32" t="s">
+        <v>372</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
+        <v>374</v>
+      </c>
+      <c r="J32" t="s">
         <v>373</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>372</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="I32" t="s">
-        <v>375</v>
-      </c>
-      <c r="J32" t="s">
-        <v>374</v>
       </c>
       <c r="K32" t="s">
         <v>13</v>
@@ -4668,45 +4755,45 @@
         <v>25</v>
       </c>
       <c r="M32" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O32" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P32" t="s">
         <v>44</v>
       </c>
       <c r="Q32" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B33" t="s">
+        <v>383</v>
+      </c>
+      <c r="C33" t="s">
         <v>384</v>
       </c>
-      <c r="C33" t="s">
-        <v>385</v>
-      </c>
       <c r="D33" t="s">
+        <v>394</v>
+      </c>
+      <c r="G33" s="9" t="s">
         <v>395</v>
       </c>
-      <c r="G33" s="9" t="s">
-        <v>396</v>
-      </c>
       <c r="H33" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I33" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J33" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K33" t="s">
         <v>13</v>
@@ -4715,39 +4802,39 @@
         <v>25</v>
       </c>
       <c r="M33" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O33" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B34" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C34" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D34" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I34" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J34" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K34" t="s">
         <v>13</v>
@@ -4756,39 +4843,39 @@
         <v>25</v>
       </c>
       <c r="M34" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O34" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B35" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C35" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D35" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I35" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J35" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K35" t="s">
         <v>13</v>
@@ -4797,39 +4884,39 @@
         <v>25</v>
       </c>
       <c r="M35" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O35" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B36" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C36" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D36" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I36" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J36" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K36" t="s">
         <v>13</v>
@@ -4838,39 +4925,39 @@
         <v>25</v>
       </c>
       <c r="M36" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O36" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B37" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C37" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D37" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I37" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J37" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K37" t="s">
         <v>13</v>
@@ -4879,39 +4966,39 @@
         <v>25</v>
       </c>
       <c r="M37" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O37" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B38" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C38" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D38" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I38" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J38" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K38" t="s">
         <v>13</v>
@@ -4920,39 +5007,39 @@
         <v>25</v>
       </c>
       <c r="M38" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O38" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B39" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C39" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D39" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I39" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J39" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K39" t="s">
         <v>13</v>
@@ -4961,39 +5048,39 @@
         <v>25</v>
       </c>
       <c r="M39" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O39" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B40" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C40" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D40" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I40" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J40" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K40" t="s">
         <v>13</v>
@@ -5002,39 +5089,39 @@
         <v>25</v>
       </c>
       <c r="M40" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O40" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B41" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C41" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D41" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I41" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J41" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K41" t="s">
         <v>13</v>
@@ -5043,39 +5130,39 @@
         <v>25</v>
       </c>
       <c r="M41" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O41" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B42" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C42" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D42" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H42" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I42" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J42" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K42" t="s">
         <v>13</v>
@@ -5084,39 +5171,39 @@
         <v>25</v>
       </c>
       <c r="M42" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O42" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B43" t="s">
+        <v>438</v>
+      </c>
+      <c r="C43" t="s">
         <v>439</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>440</v>
       </c>
-      <c r="D43" t="s">
-        <v>441</v>
-      </c>
       <c r="G43" s="9" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I43" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J43" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K43" t="s">
         <v>13</v>
@@ -5125,39 +5212,39 @@
         <v>25</v>
       </c>
       <c r="M43" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O43" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B44" t="s">
+        <v>448</v>
+      </c>
+      <c r="C44" t="s">
+        <v>439</v>
+      </c>
+      <c r="D44" t="s">
         <v>449</v>
       </c>
-      <c r="C44" t="s">
-        <v>440</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="G44" s="9" t="s">
         <v>450</v>
       </c>
-      <c r="G44" s="9" t="s">
-        <v>451</v>
-      </c>
       <c r="H44" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I44" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J44" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K44" t="s">
         <v>13</v>
@@ -5166,39 +5253,39 @@
         <v>25</v>
       </c>
       <c r="M44" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O44" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B45" t="s">
+        <v>276</v>
+      </c>
+      <c r="C45" t="s">
+        <v>439</v>
+      </c>
+      <c r="D45" t="s">
+        <v>445</v>
+      </c>
+      <c r="G45" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="C45" t="s">
-        <v>440</v>
-      </c>
-      <c r="D45" t="s">
-        <v>446</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>278</v>
-      </c>
       <c r="H45" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I45" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J45" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K45" t="s">
         <v>13</v>
@@ -5207,39 +5294,39 @@
         <v>25</v>
       </c>
       <c r="M45" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O45" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B46" t="s">
+        <v>279</v>
+      </c>
+      <c r="C46" t="s">
+        <v>439</v>
+      </c>
+      <c r="D46" t="s">
+        <v>444</v>
+      </c>
+      <c r="G46" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="C46" t="s">
-        <v>440</v>
-      </c>
-      <c r="D46" t="s">
-        <v>445</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>281</v>
-      </c>
       <c r="H46" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I46" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J46" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K46" t="s">
         <v>13</v>
@@ -5248,39 +5335,39 @@
         <v>25</v>
       </c>
       <c r="M46" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O46" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B47" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C47" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D47" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I47" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J47" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K47" t="s">
         <v>13</v>
@@ -5289,13 +5376,67 @@
         <v>25</v>
       </c>
       <c r="M47" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O47" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
         <v>458</v>
+      </c>
+      <c r="B48" s="10"/>
+      <c r="D48" t="s">
+        <v>459</v>
+      </c>
+      <c r="E48" t="s">
+        <v>67</v>
+      </c>
+      <c r="F48" t="s">
+        <v>460</v>
+      </c>
+      <c r="G48" t="s">
+        <v>461</v>
+      </c>
+      <c r="H48" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I48" t="s">
+        <v>36</v>
+      </c>
+      <c r="J48" t="s">
+        <v>11</v>
+      </c>
+      <c r="K48" t="s">
+        <v>13</v>
+      </c>
+      <c r="L48" t="s">
+        <v>25</v>
+      </c>
+      <c r="M48" t="s">
+        <v>456</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O48" t="s">
+        <v>457</v>
+      </c>
+      <c r="P48" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>462</v>
+      </c>
+      <c r="R48" t="s">
+        <v>81</v>
+      </c>
+      <c r="S48" t="s">
+        <v>463</v>
       </c>
     </row>
   </sheetData>
@@ -5329,10 +5470,10 @@
         <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>313</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>314</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>0</v>
@@ -5350,13 +5491,13 @@
         <v>2</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>14</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>15</v>
@@ -5377,10 +5518,10 @@
         <v>42</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
@@ -5388,13 +5529,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F2" t="s">
         <v>39</v>
@@ -5409,7 +5550,7 @@
         <v>46</v>
       </c>
       <c r="J2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="K2" t="s">
         <v>13</v>
@@ -5418,13 +5559,13 @@
         <v>26</v>
       </c>
       <c r="M2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N2" t="s">
         <v>40</v>
       </c>
       <c r="O2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P2" t="s">
         <v>44</v>
@@ -5438,25 +5579,25 @@
         <v>28</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H3" s="7">
         <v>0.25</v>
       </c>
       <c r="I3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K3" t="s">
         <v>13</v>
@@ -5465,45 +5606,45 @@
         <v>27</v>
       </c>
       <c r="M3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P3" t="s">
         <v>44</v>
       </c>
       <c r="Q3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" t="s">
+        <v>153</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" t="s">
-        <v>154</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="H4" s="7">
         <v>0.25</v>
       </c>
       <c r="I4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K4" t="s">
         <v>13</v>
@@ -5512,45 +5653,45 @@
         <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="O4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P4" t="s">
         <v>44</v>
       </c>
       <c r="Q4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D5" t="s">
+        <v>218</v>
+      </c>
+      <c r="E5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G5" t="s">
         <v>219</v>
-      </c>
-      <c r="E5" t="s">
-        <v>218</v>
-      </c>
-      <c r="F5" t="s">
-        <v>217</v>
-      </c>
-      <c r="G5" t="s">
-        <v>220</v>
       </c>
       <c r="H5" s="9">
         <v>0.1</v>
       </c>
       <c r="I5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K5" t="s">
         <v>13</v>
@@ -5559,42 +5700,42 @@
         <v>26</v>
       </c>
       <c r="M5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O5" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P5" t="s">
         <v>44</v>
       </c>
       <c r="Q5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G6" t="s">
+        <v>229</v>
+      </c>
+      <c r="I6" t="s">
+        <v>228</v>
+      </c>
+      <c r="J6" t="s">
         <v>230</v>
-      </c>
-      <c r="I6" t="s">
-        <v>229</v>
-      </c>
-      <c r="J6" t="s">
-        <v>231</v>
       </c>
       <c r="K6" t="s">
         <v>13</v>
@@ -5603,19 +5744,19 @@
         <v>26</v>
       </c>
       <c r="M6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="P6" t="s">
         <v>44</v>
       </c>
       <c r="Q6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>